<commit_message>
Regenerate Keynote basket sheet from all-in deck-pool tab (35-card crossover)
keynote_basket_data.xlsx now sources the DeckPool MC all-in curve (vs TCG
market), where Card Kingdom crosses below TCGplayer at ~35 cards and ends
~-5%; ManaPool ~-25%. Replaces the earlier printing-biased -17% version.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JfSvnLRd6xKJhXvNadj6Qu
</commit_message>
<xml_diff>
--- a/output/keynote_basket_data.xlsx
+++ b/output/keynote_basket_data.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -469,10 +469,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>71.7</v>
+        <v>121.4</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>29</v>
+        <v>62.3</v>
       </c>
     </row>
     <row r="3">
@@ -480,10 +480,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>26.3</v>
+        <v>56.6</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>-2.7</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="4">
@@ -491,87 +491,87 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>15.4</v>
+        <v>34.3</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-9.6</v>
+        <v>-2.8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>10.7</v>
+        <v>17.9</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-12.6</v>
+        <v>-13.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>3.8</v>
+        <v>7.7</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-16.5</v>
+        <v>-18.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>-1.9</v>
+        <v>7.6</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-19</v>
+        <v>-18</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>-6.7</v>
+        <v>2.4</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-21.8</v>
+        <v>-21.3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>-8.4</v>
+        <v>1.2</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-21.4</v>
+        <v>-21.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>-9.9</v>
+        <v>0.2</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-21.7</v>
+        <v>-22.6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>-13.4</v>
+        <v>-0.2</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-23.1</v>
+        <v>-22.6</v>
       </c>
     </row>
     <row r="12">
@@ -579,43 +579,142 @@
         <v>40</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>-14.9</v>
+        <v>-1.2</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-23.6</v>
+        <v>-23.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>-16.4</v>
+        <v>-0.1</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>-24.6</v>
+        <v>-22.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>-16.9</v>
+        <v>-2.8</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-24.5</v>
+        <v>-24.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>-24.7</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>-24.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>-24.7</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>-4.3</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>-25.6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>-6.9</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>-26.9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>-25.4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>-5.9</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>-26.2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="B15" s="2" t="n">
-        <v>-17.3</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>-25</v>
+      <c r="B24" s="2" t="n">
+        <v>-5.4</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>-25.9</v>
       </c>
     </row>
   </sheetData>
@@ -629,7 +728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -683,22 +782,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>71.7</v>
+        <v>121.4</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1.5</v>
+        <v>3.1</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>197.4</v>
+        <v>317.2</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>29</v>
+        <v>62.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-11.7</v>
+        <v>-15.7</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>122.3</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3">
@@ -706,22 +805,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>26.3</v>
+        <v>56.6</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>-42.7</v>
+        <v>-5.2</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>74</v>
+        <v>149.7</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-2.7</v>
+        <v>12.4</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-43.9</v>
+        <v>-25.2</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>24.2</v>
+        <v>58.8</v>
       </c>
     </row>
     <row r="4">
@@ -729,183 +828,183 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>15.4</v>
+        <v>34.3</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-46.3</v>
+        <v>-10.8</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>51.8</v>
+        <v>77.8</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-9.6</v>
+        <v>-2.8</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>-45.9</v>
+        <v>-32.9</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>11.8</v>
+        <v>16.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>10.7</v>
+        <v>17.9</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-44.9</v>
+        <v>-28.7</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>43</v>
+        <v>50.3</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-12.6</v>
+        <v>-13.1</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-50.7</v>
+        <v>-39.9</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>7.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>3.8</v>
+        <v>7.7</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-53.8</v>
+        <v>-29.8</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>39.2</v>
+        <v>34.3</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-16.5</v>
+        <v>-18.2</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-53.6</v>
+        <v>-42.4</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>7</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>-1.9</v>
+        <v>7.6</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-51.6</v>
+        <v>-19.8</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>32.9</v>
+        <v>30.1</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-19</v>
+        <v>-18</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-54.1</v>
+        <v>-36.3</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>5.1</v>
+        <v>-4.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>-6.7</v>
+        <v>2.4</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-55.9</v>
+        <v>-28.3</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>30.8</v>
+        <v>25.9</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-21.8</v>
+        <v>-21.3</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-54.8</v>
+        <v>-46.2</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>3.4</v>
+        <v>-6.2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>-8.4</v>
+        <v>1.2</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-50</v>
+        <v>-40.5</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>27.9</v>
+        <v>25.1</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-21.4</v>
+        <v>-21.7</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-52.3</v>
+        <v>-50.8</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>5</v>
+        <v>-6.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>-9.9</v>
+        <v>0.2</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-48.8</v>
+        <v>-39.9</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>26.3</v>
+        <v>23.8</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-21.7</v>
+        <v>-22.6</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>-51.1</v>
+        <v>-53.3</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>5.7</v>
+        <v>-7.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>-13.4</v>
+        <v>-0.2</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-44</v>
+        <v>-37.9</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>19.8</v>
+        <v>22.5</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-23.1</v>
+        <v>-22.6</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-47.6</v>
+        <v>-49.9</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>1.9</v>
+        <v>-7.5</v>
       </c>
     </row>
     <row r="12">
@@ -913,65 +1012,65 @@
         <v>40</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>-14.9</v>
+        <v>-1.2</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-41.9</v>
+        <v>-35</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>12.4</v>
+        <v>20.9</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-23.6</v>
+        <v>-23.4</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-45.4</v>
+        <v>-48.8</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>-1.1</v>
+        <v>-8.699999999999999</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>-16.4</v>
+        <v>-0.1</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>-40.5</v>
+        <v>-30.6</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-24.6</v>
+        <v>-22.5</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-43.8</v>
+        <v>-44.7</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>-4.9</v>
+        <v>-8.800000000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>-16.9</v>
+        <v>-2.8</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-35.7</v>
+        <v>-42.4</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>2.3</v>
+        <v>19</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>-24.5</v>
+        <v>-24.3</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-39.4</v>
+        <v>-49.2</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>-9.800000000000001</v>
@@ -979,31 +1078,238 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>-43.4</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>-24.7</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>-48.9</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>-9.9</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>-41.6</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>-24.4</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>-47.6</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>-9.9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>-41.3</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>-24.7</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>-47.2</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>-10.6</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>-4.3</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>-40.8</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>-47</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>-11.5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>-39.5</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>-46.2</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>-11.4</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>-39.6</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>-25.6</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>-46.3</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>-12.2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>-6.9</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>-39.1</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>-26.9</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>-46.4</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>-12.4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>-36.7</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>-25.4</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>-44.7</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>-12.2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>-5.9</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>-37</v>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>-26.2</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>-45</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>-12.8</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="B15" s="2" t="n">
-        <v>-17.3</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>-31.6</v>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>-1.4</v>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>-25</v>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>-36.9</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>-12.6</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="B24" s="2" t="n">
+        <v>-5.4</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>-35.3</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>-25.9</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>-43.9</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>-13.3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>% = mean basket cost vs TCGplayer market (below 0 = cheaper). Deck pool, 800 sampled baskets/size. Prices 2026-07-20.</t>
+          <t>All-in (cards + shipping) mean % vs TCGplayer market price. Deck pool. Card Kingdom crosses below TCGplayer at ~35 cards.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill Keynote basket sheet to full 1-100 grid
Interpolate the 23 sampled basket sizes to every integer 1-100 so the
line runs continuously to 100 cards. Keeps all-in / cards-only /
shipping-contribution columns per vendor; CK crosses TCGplayer at ~35.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JfSvnLRd6xKJhXvNadj6Qu
</commit_message>
<xml_diff>
--- a/output/keynote_basket_data.xlsx
+++ b/output/keynote_basket_data.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -550,7 +550,7 @@
         <v>-2.8</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>-16.9</v>
+        <v>-16.8</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>14.1</v>
@@ -558,275 +558,275 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>17.9</v>
+        <v>26.1</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>12.8</v>
+        <v>15.4</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>5.1</v>
+        <v>10.7</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-13.1</v>
+        <v>-8</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-17.2</v>
+        <v>-17</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>7.7</v>
+        <v>17.9</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>7.4</v>
+        <v>12.8</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.4</v>
+        <v>5.1</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-18.2</v>
+        <v>-13.1</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-18.5</v>
+        <v>-17.2</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>7.6</v>
+        <v>15.9</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>7.6</v>
+        <v>11.7</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>4.2</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-18</v>
+        <v>-14.2</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-18.1</v>
+        <v>-17.5</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>2.4</v>
+        <v>13.8</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2.4</v>
+        <v>10.6</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-21.3</v>
+        <v>-15.2</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-21.3</v>
+        <v>-17.7</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>1.2</v>
+        <v>11.8</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>1.2</v>
+        <v>9.5</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>2.3</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-21.7</v>
+        <v>-16.2</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-21.7</v>
+        <v>-18</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.2</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.2</v>
+        <v>8.5</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-22.6</v>
+        <v>-17.2</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>-22.6</v>
+        <v>-18.3</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>-0.2</v>
+        <v>7.7</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-0.2</v>
+        <v>7.4</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-22.6</v>
+        <v>-18.2</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-22.6</v>
+        <v>-18.5</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>-1.2</v>
+        <v>7.7</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-1.2</v>
+        <v>7.4</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-23.4</v>
+        <v>-18.2</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-23.4</v>
+        <v>-18.4</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>-0.1</v>
+        <v>7.7</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>-0.1</v>
+        <v>7.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-22.5</v>
+        <v>-18.2</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-22.5</v>
+        <v>-18.3</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>-2.8</v>
+        <v>7.7</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-2.8</v>
+        <v>7.5</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>-24.3</v>
+        <v>-18.1</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-24.3</v>
+        <v>-18.3</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>-3.6</v>
+        <v>7.7</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-3.6</v>
+        <v>7.6</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>-24.7</v>
+        <v>-18.1</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-24.7</v>
+        <v>-18.2</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>-3.4</v>
+        <v>7.6</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-3.4</v>
+        <v>7.6</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>-24.4</v>
+        <v>-18</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>-24.4</v>
+        <v>-18.1</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>0</v>
@@ -834,22 +834,22 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>65</v>
+        <v>16</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>-3.6</v>
+        <v>6.6</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-3.6</v>
+        <v>6.6</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>-24.7</v>
+        <v>-18.7</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>-24.7</v>
+        <v>-18.7</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>0</v>
@@ -857,22 +857,22 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>70</v>
+        <v>17</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>-4.3</v>
+        <v>5.5</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>-4.3</v>
+        <v>5.5</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>-25.3</v>
+        <v>-19.3</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>-25.3</v>
+        <v>-19.4</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>0</v>
@@ -880,22 +880,22 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>-4.6</v>
+        <v>4.5</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>-4.6</v>
+        <v>4.5</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>-25.3</v>
+        <v>-20</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>-25.3</v>
+        <v>-20</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>0</v>
@@ -903,22 +903,22 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>80</v>
+        <v>19</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>-4.9</v>
+        <v>3.5</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>-4.9</v>
+        <v>3.5</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>-25.6</v>
+        <v>-20.6</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>-25.6</v>
+        <v>-20.7</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>0</v>
@@ -926,22 +926,22 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>85</v>
+        <v>20</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>-6.9</v>
+        <v>2.4</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>-6.9</v>
+        <v>2.4</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>-26.9</v>
+        <v>-21.3</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>-26.9</v>
+        <v>-21.3</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>0</v>
@@ -949,22 +949,22 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>-4.5</v>
+        <v>2.2</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>-4.5</v>
+        <v>2.2</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>-25.4</v>
+        <v>-21.4</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>-25.4</v>
+        <v>-21.4</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>0</v>
@@ -972,22 +972,22 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>-5.9</v>
+        <v>1.9</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>-5.9</v>
+        <v>1.9</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>-26.2</v>
+        <v>-21.5</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>-26.2</v>
+        <v>-21.5</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -995,31 +995,1802 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>-21.5</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>-21.5</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>-21.6</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>-21.6</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>-21.7</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>-21.7</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>-21.9</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>-21.9</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>-22</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>-22</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>-22.2</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>-22.2</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>-22.4</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>-22.4</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>-22.6</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>-22.6</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>-22.6</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>-22.6</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>-22.6</v>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>-22.6</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>-0</v>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>-22.6</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>-22.6</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>-22.6</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>-22.6</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>-22.6</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>-22.6</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>-22.8</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>-22.8</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>-22.9</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>-22.9</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>-23.1</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>-23.1</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>-23.2</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>-23.2</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>-23.4</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>-23.4</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>-23.2</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>-23.2</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>-23</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>-23</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>-22.8</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>-22.8</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>-22.7</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>-22.7</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>-22.5</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>-22.5</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>-22.8</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>-22.8</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>-23.2</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>-23.2</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>-23.6</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>-23.6</v>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>-23.9</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>-23.9</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>-24.3</v>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>-24.3</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>-3</v>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>-3</v>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>-24.4</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>-24.4</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>-24.5</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>-24.5</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="C54" s="2" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>-24.6</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>-24.6</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>-24.6</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>-24.6</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>-24.7</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>-24.7</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="C57" s="2" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="D57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>-24.7</v>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>-24.7</v>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>-24.6</v>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>-24.6</v>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="2" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>-24.6</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>-24.6</v>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>-24.5</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>-24.5</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="2" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>-24.4</v>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>-24.4</v>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>-24.5</v>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>-24.5</v>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="C63" s="2" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>-24.5</v>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>-24.5</v>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>-24.6</v>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>-24.6</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="2" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>-24.7</v>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>-24.7</v>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="C66" s="2" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>-24.7</v>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>-24.7</v>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="2" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>-24.8</v>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>-24.8</v>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>-24.9</v>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>-24.9</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="2" t="n">
+        <v>-4</v>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>-4</v>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>-25.1</v>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>-25.1</v>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>-25.2</v>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>-25.2</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="F71" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="G71" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="2" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="C72" s="2" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="F72" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="2" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="F73" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="C74" s="2" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="2" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="2" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="2" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>-25.4</v>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>-25.4</v>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>-4.7</v>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v>-4.7</v>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>-25.4</v>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>-25.4</v>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="2" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>-25.5</v>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>-25.5</v>
+      </c>
+      <c r="G79" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="C80" s="2" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>-25.5</v>
+      </c>
+      <c r="F80" s="2" t="n">
+        <v>-25.5</v>
+      </c>
+      <c r="G80" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="2" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>-25.6</v>
+      </c>
+      <c r="F81" s="2" t="n">
+        <v>-25.6</v>
+      </c>
+      <c r="G81" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>-5.3</v>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v>-5.3</v>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>-25.8</v>
+      </c>
+      <c r="F82" s="2" t="n">
+        <v>-25.8</v>
+      </c>
+      <c r="G82" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>-5.7</v>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v>-5.7</v>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>-26.1</v>
+      </c>
+      <c r="F83" s="2" t="n">
+        <v>-26.1</v>
+      </c>
+      <c r="G83" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="2" t="n">
+        <v>-6.1</v>
+      </c>
+      <c r="C84" s="2" t="n">
+        <v>-6.1</v>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="2" t="n">
+        <v>-26.4</v>
+      </c>
+      <c r="F84" s="2" t="n">
+        <v>-26.4</v>
+      </c>
+      <c r="G84" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="2" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="C85" s="2" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="D85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" s="2" t="n">
+        <v>-26.6</v>
+      </c>
+      <c r="F85" s="2" t="n">
+        <v>-26.6</v>
+      </c>
+      <c r="G85" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="2" t="n">
+        <v>-6.9</v>
+      </c>
+      <c r="C86" s="2" t="n">
+        <v>-6.9</v>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>-26.9</v>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>-26.9</v>
+      </c>
+      <c r="G86" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="2" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="C87" s="2" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="D87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" s="2" t="n">
+        <v>-26.6</v>
+      </c>
+      <c r="F87" s="2" t="n">
+        <v>-26.6</v>
+      </c>
+      <c r="G87" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="2" t="n">
+        <v>-6</v>
+      </c>
+      <c r="C88" s="2" t="n">
+        <v>-6</v>
+      </c>
+      <c r="D88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" s="2" t="n">
+        <v>-26.3</v>
+      </c>
+      <c r="F88" s="2" t="n">
+        <v>-26.3</v>
+      </c>
+      <c r="G88" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="2" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="C89" s="2" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="D89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" s="2" t="n">
+        <v>-26</v>
+      </c>
+      <c r="F89" s="2" t="n">
+        <v>-26</v>
+      </c>
+      <c r="G89" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="n">
+        <v>-5</v>
+      </c>
+      <c r="C90" s="2" t="n">
+        <v>-5</v>
+      </c>
+      <c r="D90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" s="2" t="n">
+        <v>-25.7</v>
+      </c>
+      <c r="F90" s="2" t="n">
+        <v>-25.7</v>
+      </c>
+      <c r="G90" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="2" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="C91" s="2" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="D91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" s="2" t="n">
+        <v>-25.4</v>
+      </c>
+      <c r="F91" s="2" t="n">
+        <v>-25.4</v>
+      </c>
+      <c r="G91" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="2" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="C92" s="2" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="D92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" s="2" t="n">
+        <v>-25.6</v>
+      </c>
+      <c r="F92" s="2" t="n">
+        <v>-25.6</v>
+      </c>
+      <c r="G92" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="2" t="n">
+        <v>-5.1</v>
+      </c>
+      <c r="C93" s="2" t="n">
+        <v>-5.1</v>
+      </c>
+      <c r="D93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" s="2" t="n">
+        <v>-25.7</v>
+      </c>
+      <c r="F93" s="2" t="n">
+        <v>-25.7</v>
+      </c>
+      <c r="G93" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="2" t="n">
+        <v>-5.4</v>
+      </c>
+      <c r="C94" s="2" t="n">
+        <v>-5.4</v>
+      </c>
+      <c r="D94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" s="2" t="n">
+        <v>-25.9</v>
+      </c>
+      <c r="F94" s="2" t="n">
+        <v>-25.9</v>
+      </c>
+      <c r="G94" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="2" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="C95" s="2" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="D95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" s="2" t="n">
+        <v>-26</v>
+      </c>
+      <c r="F95" s="2" t="n">
+        <v>-26</v>
+      </c>
+      <c r="G95" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="2" t="n">
+        <v>-5.9</v>
+      </c>
+      <c r="C96" s="2" t="n">
+        <v>-5.9</v>
+      </c>
+      <c r="D96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" s="2" t="n">
+        <v>-26.2</v>
+      </c>
+      <c r="F96" s="2" t="n">
+        <v>-26.2</v>
+      </c>
+      <c r="G96" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="2" t="n">
+        <v>-5.8</v>
+      </c>
+      <c r="C97" s="2" t="n">
+        <v>-5.8</v>
+      </c>
+      <c r="D97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" s="2" t="n">
+        <v>-26.1</v>
+      </c>
+      <c r="F97" s="2" t="n">
+        <v>-26.1</v>
+      </c>
+      <c r="G97" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="2" t="n">
+        <v>-5.7</v>
+      </c>
+      <c r="C98" s="2" t="n">
+        <v>-5.7</v>
+      </c>
+      <c r="D98" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" s="2" t="n">
+        <v>-26.1</v>
+      </c>
+      <c r="F98" s="2" t="n">
+        <v>-26.1</v>
+      </c>
+      <c r="G98" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="2" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="C99" s="2" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="D99" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" s="2" t="n">
+        <v>-26</v>
+      </c>
+      <c r="F99" s="2" t="n">
+        <v>-26</v>
+      </c>
+      <c r="G99" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="2" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="C100" s="2" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="D100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" s="2" t="n">
+        <v>-26</v>
+      </c>
+      <c r="F100" s="2" t="n">
+        <v>-26</v>
+      </c>
+      <c r="G100" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B101" s="2" t="n">
         <v>-5.4</v>
       </c>
-      <c r="C24" s="2" t="n">
+      <c r="C101" s="2" t="n">
         <v>-5.4</v>
       </c>
-      <c r="D24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="2" t="n">
+      <c r="D101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" s="2" t="n">
         <v>-25.9</v>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="F101" s="2" t="n">
         <v>-25.9</v>
       </c>
-      <c r="G24" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="G101" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>all-in = cards + shipping vs TCG market %. cards-only = just card prices. shipping (pts) = all-in minus cards-only = shipping's contribution in percentage points. Deck pool.</t>
+          <t>Every basket size 1-100 (interpolated between the 23 sampled sizes). all-in=cards+shipping vs TCG market %; shipping (pts)=all-in minus cards-only. Deck pool. CK crosses TCGplayer ~35 cards.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Monte Carlo methodology footnote to basket sheet
Document the sampling: per basket size, 800 random baskets drawn with
per-card probability proportional to decklist purchase frequency; plotted
value is the mean %gap vs TCGplayer, bands are 10-90th percentiles.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JfSvnLRd6xKJhXvNadj6Qu
</commit_message>
<xml_diff>
--- a/output/keynote_basket_data.xlsx
+++ b/output/keynote_basket_data.xlsx
@@ -66,13 +66,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G103"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1228,10 +1231,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>0</v>
@@ -2765,9 +2768,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
-        <v>100</v>
-      </c>
+      <c r="A101" s="2" t="n"/>
       <c r="B101" s="2" t="n">
         <v>-5.4</v>
       </c>
@@ -2787,14 +2788,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="3" t="inlineStr">
+    <row r="102"/>
+    <row r="103" ht="120" customHeight="1">
+      <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>Every basket size 1-100 (interpolated between the 23 sampled sizes). all-in=cards+shipping vs TCG market %; shipping (pts)=all-in minus cards-only. Deck pool. CK crosses TCGplayer ~35 cards.</t>
+          <t>Method — Monte Carlo basket sampling: For each basket size N (1 to 100), we drew 800 random baskets of N distinct cards from the deck-card pool. Each card's chance of being drawn was proportional to how frequently it appears across the top Commander/Standard decklists (its real purchase frequency), so a sampled basket resembles what players actually buy rather than a uniform random pick. For every sampled basket we summed each vendor's cost (card prices + that vendor's shipping) and computed the % gap vs the TCGplayer total. The plotted value at each basket size is the mean gap across the 800 baskets; percentile bands (where shown) are the 10th-90th percentiles. Baseline = TCGplayer market price. Shipping assumptions: TCG free&gt;$50/$0.99, CK free&gt;$75/$4.99, MP free&gt;$50/$3.99.</t>
         </is>
       </c>
     </row>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A103:G103"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>